<commit_message>
Update tracker: mark Phase 2-3 tasks done, add tasks 76-82
Done: #6 BPM, #7 Key, #10 Volume, #11 Mono, #12 FilterBank, #15 LiveSpec,
      #16 PhaseMeter, #17 LUFS meter, #18 Vectorscope, #24 Canvas DPR,
      #53 LUFS ST bug, #74 M/S live, #75 M/S static
New:  #76 GitHub Actions, #77 Electron, #78 Waveform zoom,
      #79 BPM verification (todo), #80 PR orphan branch fix (todo),
      #81 App icon (todo), #82 Vectorscope fftSize QA (todo)

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/mix-analyzer-tracker.xlsx
+++ b/mix-analyzer-tracker.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="16">
+  <fonts count="18">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -103,8 +103,16 @@
       <color rgb="005B4FA0"/>
       <sz val="9.5"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00276221"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="009C6500"/>
+    </font>
   </fonts>
-  <fills count="9">
+  <fills count="11">
     <fill>
       <patternFill/>
     </fill>
@@ -144,6 +152,16 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FFF8E8"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C6EFCE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFEB9C"/>
       </patternFill>
     </fill>
   </fills>
@@ -217,7 +235,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="34">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -303,6 +321,11 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="16" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="9" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="17" fillId="10" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -668,7 +691,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G108"/>
+  <dimension ref="A1:G117"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -919,9 +942,9 @@
           <t>BPM detection (onset + autocorrelation)</t>
         </is>
       </c>
-      <c r="D8" s="19" t="inlineStr">
-        <is>
-          <t>Todo</t>
+      <c r="D8" s="31" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="E8" s="17" t="inlineStr">
@@ -931,7 +954,7 @@
       </c>
       <c r="F8" s="15" t="inlineStr">
         <is>
-          <t>LP filter → onset strength → autocorrelation → peak pick in 60-200 BPM. Windowed for tempo changes (8-16 bar sliding). Beat grid markers.</t>
+          <t>Enhanced autocorrelation: hop=256, harmonic scoring (AC[lag]+0.5*AC[2lag]+...), octave correction fixed. Verified 144 BPM on test track.</t>
         </is>
       </c>
       <c r="G8" s="20" t="inlineStr">
@@ -954,9 +977,9 @@
           <t>Key detection (chromagram + Krumhansl profiles)</t>
         </is>
       </c>
-      <c r="D9" s="19" t="inlineStr">
-        <is>
-          <t>Todo</t>
+      <c r="D9" s="31" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="E9" s="18" t="inlineStr">
@@ -966,7 +989,7 @@
       </c>
       <c r="F9" s="9" t="inlineStr">
         <is>
-          <t>FFT → 12 pitch classes (octave fold) → correlate all 24 major/minor profiles. Windowed for key changes. Camelot wheel output.</t>
+          <t>Chromagram via FFT bin-&gt;pitch class + Krumhansl-Kessler Pearson correlation. Returns key/root/mode/confidence/chroma.</t>
         </is>
       </c>
       <c r="G9" s="21" t="inlineStr">
@@ -1072,7 +1095,7 @@
           <t>Volume control (GainNode)</t>
         </is>
       </c>
-      <c r="D13" s="19" t="inlineStr">
+      <c r="D13" s="31" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
@@ -1084,7 +1107,7 @@
       </c>
       <c r="F13" s="15" t="inlineStr">
         <is>
-          <t>Insert GainNode between source and destination. Slider in toolbar.</t>
+          <t>GainNode in audio output chain. Volume slider 0-100% in transport bar.</t>
         </is>
       </c>
       <c r="G13" s="22" t="inlineStr">
@@ -1107,7 +1130,7 @@
           <t>Mono preview toggle</t>
         </is>
       </c>
-      <c r="D14" s="19" t="inlineStr">
+      <c r="D14" s="31" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
@@ -1119,7 +1142,7 @@
       </c>
       <c r="F14" s="9" t="inlineStr">
         <is>
-          <t>ChannelMerger to sum L+R. Critical for checking mono compatibility.</t>
+          <t>ChannelMerger to sum L+R. MONO button in transport bar. Restarts playback to rebuild audio graph.</t>
         </is>
       </c>
       <c r="G14" s="23" t="inlineStr">
@@ -1142,7 +1165,7 @@
           <t>3-band filter bank (live analysis path)</t>
         </is>
       </c>
-      <c r="D15" s="19" t="inlineStr">
+      <c r="D15" s="31" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
@@ -1154,7 +1177,7 @@
       </c>
       <c r="F15" s="15" t="inlineStr">
         <is>
-          <t>Phase 2: 3-band BiquadFilter bank with 6 AnalyserNodes (LP 200Hz / BP 200-4kHz / HP 4kHz). Parallel analysis path, no effect on audio output. Built in playFrom(), torn down in killSource().</t>
+          <t>LP 200Hz / BP 200-4kHz / HP 4kHz per channel = 6 AnalyserNodes. Wideband L/R added for vectorscope + M/S.</t>
         </is>
       </c>
       <c r="G15" s="20" t="inlineStr">
@@ -1260,7 +1283,7 @@
           <t>Live spectrum analyzer (Canvas)</t>
         </is>
       </c>
-      <c r="D19" s="19" t="inlineStr">
+      <c r="D19" s="31" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
@@ -1272,7 +1295,7 @@
       </c>
       <c r="F19" s="9" t="inlineStr">
         <is>
-          <t>Phase 2: Canvas 2D live spectrum at 60fps via requestAnimationFrame. getFloatFrequencyData() → log-freq X, dB Y. Band-colored fills (Low/Mid/High). Slope compensation. Glow + main line. Freq labels. Sits above waveform.</t>
+          <t>Line + spectrograph modes combined MiniMeters-style (spectrograph scrolls in BG, live curve on top). M/S toggle works in both modes.</t>
         </is>
       </c>
       <c r="G19" s="24" t="inlineStr">
@@ -1295,7 +1318,7 @@
           <t>3-band stereo phase meter</t>
         </is>
       </c>
-      <c r="D20" s="19" t="inlineStr">
+      <c r="D20" s="31" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
@@ -1307,7 +1330,7 @@
       </c>
       <c r="F20" s="15" t="inlineStr">
         <is>
-          <t>Per-band L/R correlation from filter bank AnalyserNodes. Three bars: LOW/MID/HIGH. Dot position = correlation (-1 to +1). Green/yellow/red coloring. Updates 30fps. Sits beside LUFS meter.</t>
+          <t>Pearson correlation per band + stereo width. Dot indicator maps -1..+1 to L..R axis.</t>
         </is>
       </c>
       <c r="G20" s="20" t="inlineStr">
@@ -1330,7 +1353,7 @@
           <t>Live LUFS meter (momentary + short-term)</t>
         </is>
       </c>
-      <c r="D21" s="19" t="inlineStr">
+      <c r="D21" s="31" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
@@ -1342,7 +1365,7 @@
       </c>
       <c r="F21" s="9" t="inlineStr">
         <is>
-          <t>K-weighted real-time from AnalyserNode data. Vertical bars: momentary (400ms) + short-term (3s). Color zones. Target line from prefs. Sits beside stereo phase.</t>
+          <t>Momentary (400ms RMS) + short-term (3s rolling avg) bars. Peak hold with slow decay.</t>
         </is>
       </c>
       <c r="G21" s="21" t="inlineStr">
@@ -1365,9 +1388,9 @@
           <t>Live vectorscope (Canvas)</t>
         </is>
       </c>
-      <c r="D22" s="19" t="inlineStr">
-        <is>
-          <t>Todo</t>
+      <c r="D22" s="31" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="E22" s="12" t="inlineStr">
@@ -1377,7 +1400,7 @@
       </c>
       <c r="F22" s="15" t="inlineStr">
         <is>
-          <t>Real-time Lissajous during playback. Canvas-based. Optional multiband coloring (RGB by L/M/H).</t>
+          <t>Real-time M/S Lissajous from wideband L/R analysers. Multiband RGB coloring: red=Low, green=Mid, blue=High per sample.</t>
         </is>
       </c>
       <c r="G22" s="20" t="inlineStr">
@@ -1588,7 +1611,7 @@
           <t>Canvas migration for waveform</t>
         </is>
       </c>
-      <c r="D29" s="19" t="inlineStr">
+      <c r="D29" s="31" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
@@ -1600,7 +1623,7 @@
       </c>
       <c r="F29" s="15" t="inlineStr">
         <is>
-          <t>Phase 2: Migrated ~600 SVG elements to Canvas 2D. Two-layer approach: static waveform canvas + overlay canvas for playhead. drawWaveCanvas() for spectral/uniform modes, drawOverlay() for playhead.</t>
+          <t>setupCanvas() helper: DPR-aware scaling on all 5 draw functions. CSS height replaces HTML width/height attrs.</t>
         </is>
       </c>
       <c r="G29" s="20" t="inlineStr">
@@ -2694,9 +2717,9 @@
           <t>LUFS short-term: only final 3s window</t>
         </is>
       </c>
-      <c r="D65" s="19" t="inlineStr">
-        <is>
-          <t>Todo</t>
+      <c r="D65" s="31" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="E65" s="5" t="inlineStr">
@@ -2706,7 +2729,7 @@
       </c>
       <c r="F65" s="9" t="inlineStr">
         <is>
-          <t>Should track max short-term across full track.</t>
+          <t>Fixed: reuses stBlocks from LRA loop, takes Math.max(...absGated). Was only measuring tail 3s window.</t>
         </is>
       </c>
       <c r="G65" s="23" t="inlineStr">
@@ -4167,6 +4190,321 @@
       <c r="G108" t="inlineStr">
         <is>
           <t>Small</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="n">
+        <v>76</v>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>Infrastructure</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>GitHub Actions cross-platform build (Win + Mac)</t>
+        </is>
+      </c>
+      <c r="D109" s="32" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F109" t="inlineStr">
+        <is>
+          <t>build.yml: push tag v* triggers windows-latest (.exe NSIS+portable) + macos-latest (.dmg universal). Artifacts uploaded.</t>
+        </is>
+      </c>
+      <c r="G109" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="n">
+        <v>77</v>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>Infrastructure</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>Electron desktop app wrapper</t>
+        </is>
+      </c>
+      <c r="D110" s="32" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F110" t="inlineStr">
+        <is>
+          <t>electron/main.cjs (CJS, renamed from .js to fix type:module conflict). electron-builder: NSIS installer + portable .exe. release/ gitignored.</t>
+        </is>
+      </c>
+      <c r="G110" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="n">
+        <v>78</v>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>Display</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>Waveform zoom + scroll</t>
+        </is>
+      </c>
+      <c r="D111" s="32" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F111" t="inlineStr">
+        <is>
+          <t>1x/2x/4x/8x zoom buttons + mouse wheel. Scroll slider. Auto-follows playhead when zoomed. Mini-map strip at waveform bottom. Seek accounts for zoom window.</t>
+        </is>
+      </c>
+      <c r="G111" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="n">
+        <v>79</v>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>Bugs</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>Verify BPM accuracy across multiple tracks</t>
+        </is>
+      </c>
+      <c r="D112" s="33" t="inlineStr">
+        <is>
+          <t>Todo</t>
+        </is>
+      </c>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="F112" t="inlineStr">
+        <is>
+          <t>Tested on one track (144 BPM confirmed). Need 4-5 more tracks at varied tempos (90, 120, 170+ BPM) to validate enhanced AC algorithm.</t>
+        </is>
+      </c>
+      <c r="G112" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="n">
+        <v>80</v>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>Bugs</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>PR creation blocked: orphan branch history</t>
+        </is>
+      </c>
+      <c r="D113" s="33" t="inlineStr">
+        <is>
+          <t>Todo</t>
+        </is>
+      </c>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="F113" t="inlineStr">
+        <is>
+          <t>main and feature branch created as unrelated orphans. GitHub rejects PR. Fix: rebase feature commits onto proper main scaffold before opening PR. Repo: github.com/rossxo-m/MixAnalyzer</t>
+        </is>
+      </c>
+      <c r="G113" t="inlineStr">
+        <is>
+          <t>Small</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="n">
+        <v>81</v>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>Infrastructure</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>App icon (icon.ico + icon.icns)</t>
+        </is>
+      </c>
+      <c r="D114" s="33" t="inlineStr">
+        <is>
+          <t>Todo</t>
+        </is>
+      </c>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="F114" t="inlineStr">
+        <is>
+          <t>electron-builder uses default Electron icon. Need 256x256 .ico (Windows) and 512x512 .icns (macOS). Can generate from single 1024x1024 PNG.</t>
+        </is>
+      </c>
+      <c r="G114" t="inlineStr">
+        <is>
+          <t>Small</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="n">
+        <v>82</v>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>Bugs</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>Vectorscope multiband band/wideband fftSize mismatch</t>
+        </is>
+      </c>
+      <c r="D115" s="33" t="inlineStr">
+        <is>
+          <t>Todo</t>
+        </is>
+      </c>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F115" t="inlineStr">
+        <is>
+          <t>Band analysers fftSize=512, wideband fftSize=4096. Stride mapping (Math.round(bufSize/bandBufSize)) used but needs visual QA — coloring may be slightly misaligned at transients.</t>
+        </is>
+      </c>
+      <c r="G115" t="inlineStr">
+        <is>
+          <t>Small</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="n">
+        <v>74</v>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>Live Viz</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>M/S mode for live spectrum</t>
+        </is>
+      </c>
+      <c r="D116" s="32" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F116" t="inlineStr">
+        <is>
+          <t>M/S is a toggle button (not a mode). Works alongside line and spectrograph modes. lFreq/rFreq -&gt; M=(L+R)/2, S=(R-L)/2 in dB domain. Mid=blue, Side=orange.</t>
+        </is>
+      </c>
+      <c r="G116" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="n">
+        <v>75</v>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>Analysis</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>M/S mode for static spectrum</t>
+        </is>
+      </c>
+      <c r="D117" s="32" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E117" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F117" t="inlineStr">
+        <is>
+          <t>computeSpectrum returns spectrumPointsS (Side channel FFT). SpectrumDisplay has M/S toggle. Slope compensation applied to both M and S curves.</t>
+        </is>
+      </c>
+      <c r="G117" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
     </row>

</xml_diff>